<commit_message>
auto: actualizar indicadores adelantados 2026-06-15
</commit_message>
<xml_diff>
--- a/datos/indicadores_adelantados/cemento/produccion_cemento_depto_1991_2026.xlsx
+++ b/datos/indicadores_adelantados/cemento/produccion_cemento_depto_1991_2026.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="5" rupBuild="14420"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="24332"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="d:\gcondorenz\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="U:\1. Página Web\2026 - 06. Junio\Cemento 04-2026\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FF863199-B5E4-425C-A30C-26E066413708}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12330"/>
+    <workbookView xWindow="28680" yWindow="270" windowWidth="25440" windowHeight="15270" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="C1" sheetId="1" r:id="rId1"/>
@@ -24,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="438" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="439" uniqueCount="27">
   <si>
     <t>Enero</t>
   </si>
@@ -119,28 +120,6 @@
     </r>
   </si>
   <si>
-    <r>
-      <t xml:space="preserve">             </t>
-    </r>
-    <r>
-      <rPr>
-        <vertAlign val="superscript"/>
-        <sz val="9"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>(p)</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> : Preliminar</t>
-    </r>
-  </si>
-  <si>
     <t>Fuente: Empresas productoras de cemento</t>
   </si>
   <si>
@@ -161,16 +140,38 @@
   <si>
     <t>BOLIVIA: PRODUCCIÓN DE CEMENTO POR DEPARTAMENTO SEGÚN AÑO Y MES, 1991 - 2026</t>
   </si>
+  <si>
+    <r>
+      <t xml:space="preserve">             </t>
+    </r>
+    <r>
+      <rPr>
+        <vertAlign val="superscript"/>
+        <sz val="8"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>(p)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> : Preliminar</t>
+    </r>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
     <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="164" formatCode="#,##0.00000"/>
   </numFmts>
-  <fonts count="15" x14ac:knownFonts="1">
+  <fonts count="16" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -262,8 +263,13 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="8"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
       <vertAlign val="superscript"/>
-      <sz val="9"/>
+      <sz val="8"/>
       <name val="Arial"/>
       <family val="2"/>
     </font>
@@ -396,7 +402,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="13" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -460,14 +466,15 @@
     <xf numFmtId="3" fontId="7" fillId="5" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="3" fontId="8" fillId="3" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
     <xf numFmtId="43" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="3" fontId="8" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="3" fontId="8" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
   </cellXfs>
@@ -608,6 +615,23 @@
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri" panose="020F0502020204030204"/>
@@ -643,6 +667,23 @@
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -818,7 +859,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="C1:S503"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
@@ -1339,7 +1380,7 @@
     <row r="1" spans="3:19" ht="75.75" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="2" spans="3:19" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C2" s="12" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="D2" s="12"/>
       <c r="E2" s="12"/>
@@ -1422,14 +1463,14 @@
       <c r="J6" s="17">
         <v>587056.95000000007</v>
       </c>
-      <c r="L6" s="26"/>
-      <c r="M6" s="26"/>
-      <c r="N6" s="26"/>
-      <c r="O6" s="26"/>
-      <c r="P6" s="26"/>
-      <c r="Q6" s="26"/>
-      <c r="R6" s="26"/>
-      <c r="S6" s="26"/>
+      <c r="L6" s="25"/>
+      <c r="M6" s="25"/>
+      <c r="N6" s="25"/>
+      <c r="O6" s="25"/>
+      <c r="P6" s="25"/>
+      <c r="Q6" s="25"/>
+      <c r="R6" s="25"/>
+      <c r="S6" s="25"/>
     </row>
     <row r="7" spans="3:19" s="3" customFormat="1" ht="12.75" x14ac:dyDescent="0.2">
       <c r="C7" s="21" t="s">
@@ -1778,14 +1819,14 @@
       <c r="J20" s="17">
         <v>649643.79</v>
       </c>
-      <c r="L20" s="26"/>
-      <c r="M20" s="26"/>
-      <c r="N20" s="26"/>
-      <c r="O20" s="26"/>
-      <c r="P20" s="26"/>
-      <c r="Q20" s="26"/>
-      <c r="R20" s="26"/>
-      <c r="S20" s="26"/>
+      <c r="L20" s="25"/>
+      <c r="M20" s="25"/>
+      <c r="N20" s="25"/>
+      <c r="O20" s="25"/>
+      <c r="P20" s="25"/>
+      <c r="Q20" s="25"/>
+      <c r="R20" s="25"/>
+      <c r="S20" s="25"/>
     </row>
     <row r="21" spans="3:19" s="3" customFormat="1" ht="12.75" x14ac:dyDescent="0.2">
       <c r="C21" s="21" t="s">
@@ -2134,14 +2175,14 @@
       <c r="J34" s="17">
         <v>717607.41</v>
       </c>
-      <c r="L34" s="26"/>
-      <c r="M34" s="26"/>
-      <c r="N34" s="26"/>
-      <c r="O34" s="26"/>
-      <c r="P34" s="26"/>
-      <c r="Q34" s="26"/>
-      <c r="R34" s="26"/>
-      <c r="S34" s="26"/>
+      <c r="L34" s="25"/>
+      <c r="M34" s="25"/>
+      <c r="N34" s="25"/>
+      <c r="O34" s="25"/>
+      <c r="P34" s="25"/>
+      <c r="Q34" s="25"/>
+      <c r="R34" s="25"/>
+      <c r="S34" s="25"/>
     </row>
     <row r="35" spans="3:19" s="3" customFormat="1" ht="12.75" x14ac:dyDescent="0.2">
       <c r="C35" s="21" t="s">
@@ -2490,14 +2531,14 @@
       <c r="J48" s="17">
         <v>776301.62999999989</v>
       </c>
-      <c r="L48" s="26"/>
-      <c r="M48" s="26"/>
-      <c r="N48" s="26"/>
-      <c r="O48" s="26"/>
-      <c r="P48" s="26"/>
-      <c r="Q48" s="26"/>
-      <c r="R48" s="26"/>
-      <c r="S48" s="26"/>
+      <c r="L48" s="25"/>
+      <c r="M48" s="25"/>
+      <c r="N48" s="25"/>
+      <c r="O48" s="25"/>
+      <c r="P48" s="25"/>
+      <c r="Q48" s="25"/>
+      <c r="R48" s="25"/>
+      <c r="S48" s="25"/>
     </row>
     <row r="49" spans="3:19" s="3" customFormat="1" ht="12.75" x14ac:dyDescent="0.2">
       <c r="C49" s="21" t="s">
@@ -2846,14 +2887,14 @@
       <c r="J62" s="17">
         <v>892430.95000000007</v>
       </c>
-      <c r="L62" s="26"/>
-      <c r="M62" s="26"/>
-      <c r="N62" s="26"/>
-      <c r="O62" s="26"/>
-      <c r="P62" s="26"/>
-      <c r="Q62" s="26"/>
-      <c r="R62" s="26"/>
-      <c r="S62" s="26"/>
+      <c r="L62" s="25"/>
+      <c r="M62" s="25"/>
+      <c r="N62" s="25"/>
+      <c r="O62" s="25"/>
+      <c r="P62" s="25"/>
+      <c r="Q62" s="25"/>
+      <c r="R62" s="25"/>
+      <c r="S62" s="25"/>
     </row>
     <row r="63" spans="3:19" s="3" customFormat="1" ht="12.75" x14ac:dyDescent="0.2">
       <c r="C63" s="21" t="s">
@@ -3202,14 +3243,14 @@
       <c r="J76" s="17">
         <v>900956.8</v>
       </c>
-      <c r="L76" s="26"/>
-      <c r="M76" s="26"/>
-      <c r="N76" s="26"/>
-      <c r="O76" s="26"/>
-      <c r="P76" s="26"/>
-      <c r="Q76" s="26"/>
-      <c r="R76" s="26"/>
-      <c r="S76" s="26"/>
+      <c r="L76" s="25"/>
+      <c r="M76" s="25"/>
+      <c r="N76" s="25"/>
+      <c r="O76" s="25"/>
+      <c r="P76" s="25"/>
+      <c r="Q76" s="25"/>
+      <c r="R76" s="25"/>
+      <c r="S76" s="25"/>
     </row>
     <row r="77" spans="3:19" s="3" customFormat="1" ht="12.75" x14ac:dyDescent="0.2">
       <c r="C77" s="21" t="s">
@@ -3558,14 +3599,14 @@
       <c r="J90" s="17">
         <v>1047951.0700000001</v>
       </c>
-      <c r="L90" s="26"/>
-      <c r="M90" s="26"/>
-      <c r="N90" s="26"/>
-      <c r="O90" s="26"/>
-      <c r="P90" s="26"/>
-      <c r="Q90" s="26"/>
-      <c r="R90" s="26"/>
-      <c r="S90" s="26"/>
+      <c r="L90" s="25"/>
+      <c r="M90" s="25"/>
+      <c r="N90" s="25"/>
+      <c r="O90" s="25"/>
+      <c r="P90" s="25"/>
+      <c r="Q90" s="25"/>
+      <c r="R90" s="25"/>
+      <c r="S90" s="25"/>
     </row>
     <row r="91" spans="3:19" s="3" customFormat="1" ht="12.75" x14ac:dyDescent="0.2">
       <c r="C91" s="21" t="s">
@@ -3914,14 +3955,14 @@
       <c r="J104" s="17">
         <v>1166511.1599999997</v>
       </c>
-      <c r="L104" s="26"/>
-      <c r="M104" s="26"/>
-      <c r="N104" s="26"/>
-      <c r="O104" s="26"/>
-      <c r="P104" s="26"/>
-      <c r="Q104" s="26"/>
-      <c r="R104" s="26"/>
-      <c r="S104" s="26"/>
+      <c r="L104" s="25"/>
+      <c r="M104" s="25"/>
+      <c r="N104" s="25"/>
+      <c r="O104" s="25"/>
+      <c r="P104" s="25"/>
+      <c r="Q104" s="25"/>
+      <c r="R104" s="25"/>
+      <c r="S104" s="25"/>
     </row>
     <row r="105" spans="3:19" s="3" customFormat="1" ht="12.75" x14ac:dyDescent="0.2">
       <c r="C105" s="21" t="s">
@@ -4270,14 +4311,14 @@
       <c r="J118" s="17">
         <v>1201274.32</v>
       </c>
-      <c r="L118" s="26"/>
-      <c r="M118" s="26"/>
-      <c r="N118" s="26"/>
-      <c r="O118" s="26"/>
-      <c r="P118" s="26"/>
-      <c r="Q118" s="26"/>
-      <c r="R118" s="26"/>
-      <c r="S118" s="26"/>
+      <c r="L118" s="25"/>
+      <c r="M118" s="25"/>
+      <c r="N118" s="25"/>
+      <c r="O118" s="25"/>
+      <c r="P118" s="25"/>
+      <c r="Q118" s="25"/>
+      <c r="R118" s="25"/>
+      <c r="S118" s="25"/>
     </row>
     <row r="119" spans="3:19" ht="12.75" x14ac:dyDescent="0.2">
       <c r="C119" s="21" t="s">
@@ -4730,14 +4771,14 @@
       <c r="J132" s="17">
         <v>1071941</v>
       </c>
-      <c r="L132" s="26"/>
-      <c r="M132" s="26"/>
-      <c r="N132" s="26"/>
-      <c r="O132" s="26"/>
-      <c r="P132" s="26"/>
-      <c r="Q132" s="26"/>
-      <c r="R132" s="26"/>
-      <c r="S132" s="26"/>
+      <c r="L132" s="25"/>
+      <c r="M132" s="25"/>
+      <c r="N132" s="25"/>
+      <c r="O132" s="25"/>
+      <c r="P132" s="25"/>
+      <c r="Q132" s="25"/>
+      <c r="R132" s="25"/>
+      <c r="S132" s="25"/>
     </row>
     <row r="133" spans="3:19" ht="12.75" x14ac:dyDescent="0.2">
       <c r="C133" s="21" t="s">
@@ -5190,14 +5231,14 @@
       <c r="J146" s="17">
         <v>982543.11</v>
       </c>
-      <c r="L146" s="26"/>
-      <c r="M146" s="26"/>
-      <c r="N146" s="26"/>
-      <c r="O146" s="26"/>
-      <c r="P146" s="26"/>
-      <c r="Q146" s="26"/>
-      <c r="R146" s="26"/>
-      <c r="S146" s="26"/>
+      <c r="L146" s="25"/>
+      <c r="M146" s="25"/>
+      <c r="N146" s="25"/>
+      <c r="O146" s="25"/>
+      <c r="P146" s="25"/>
+      <c r="Q146" s="25"/>
+      <c r="R146" s="25"/>
+      <c r="S146" s="25"/>
     </row>
     <row r="147" spans="3:19" ht="12.75" x14ac:dyDescent="0.2">
       <c r="C147" s="21" t="s">
@@ -5650,14 +5691,14 @@
       <c r="J160" s="17">
         <v>1010445.99</v>
       </c>
-      <c r="L160" s="26"/>
-      <c r="M160" s="26"/>
-      <c r="N160" s="26"/>
-      <c r="O160" s="26"/>
-      <c r="P160" s="26"/>
-      <c r="Q160" s="26"/>
-      <c r="R160" s="26"/>
-      <c r="S160" s="26"/>
+      <c r="L160" s="25"/>
+      <c r="M160" s="25"/>
+      <c r="N160" s="25"/>
+      <c r="O160" s="25"/>
+      <c r="P160" s="25"/>
+      <c r="Q160" s="25"/>
+      <c r="R160" s="25"/>
+      <c r="S160" s="25"/>
     </row>
     <row r="161" spans="3:19" ht="12.75" x14ac:dyDescent="0.2">
       <c r="C161" s="21" t="s">
@@ -6110,14 +6151,14 @@
       <c r="J174" s="17">
         <v>1138146.21</v>
       </c>
-      <c r="L174" s="26"/>
-      <c r="M174" s="26"/>
-      <c r="N174" s="26"/>
-      <c r="O174" s="26"/>
-      <c r="P174" s="26"/>
-      <c r="Q174" s="26"/>
-      <c r="R174" s="26"/>
-      <c r="S174" s="26"/>
+      <c r="L174" s="25"/>
+      <c r="M174" s="25"/>
+      <c r="N174" s="25"/>
+      <c r="O174" s="25"/>
+      <c r="P174" s="25"/>
+      <c r="Q174" s="25"/>
+      <c r="R174" s="25"/>
+      <c r="S174" s="25"/>
     </row>
     <row r="175" spans="3:19" ht="12.75" x14ac:dyDescent="0.2">
       <c r="C175" s="21" t="s">
@@ -6570,14 +6611,14 @@
       <c r="J188" s="17">
         <v>1276411.5103322999</v>
       </c>
-      <c r="L188" s="26"/>
-      <c r="M188" s="26"/>
-      <c r="N188" s="26"/>
-      <c r="O188" s="26"/>
-      <c r="P188" s="26"/>
-      <c r="Q188" s="26"/>
-      <c r="R188" s="26"/>
-      <c r="S188" s="26"/>
+      <c r="L188" s="25"/>
+      <c r="M188" s="25"/>
+      <c r="N188" s="25"/>
+      <c r="O188" s="25"/>
+      <c r="P188" s="25"/>
+      <c r="Q188" s="25"/>
+      <c r="R188" s="25"/>
+      <c r="S188" s="25"/>
     </row>
     <row r="189" spans="3:19" ht="12.75" x14ac:dyDescent="0.2">
       <c r="C189" s="21" t="s">
@@ -7030,14 +7071,14 @@
       <c r="J202" s="17">
         <v>1439951.1600000001</v>
       </c>
-      <c r="L202" s="26"/>
-      <c r="M202" s="26"/>
-      <c r="N202" s="26"/>
-      <c r="O202" s="26"/>
-      <c r="P202" s="26"/>
-      <c r="Q202" s="26"/>
-      <c r="R202" s="26"/>
-      <c r="S202" s="26"/>
+      <c r="L202" s="25"/>
+      <c r="M202" s="25"/>
+      <c r="N202" s="25"/>
+      <c r="O202" s="25"/>
+      <c r="P202" s="25"/>
+      <c r="Q202" s="25"/>
+      <c r="R202" s="25"/>
+      <c r="S202" s="25"/>
     </row>
     <row r="203" spans="3:19" ht="12.75" x14ac:dyDescent="0.2">
       <c r="C203" s="21" t="s">
@@ -7490,14 +7531,14 @@
       <c r="J216" s="17">
         <v>1636078.7199999997</v>
       </c>
-      <c r="L216" s="26"/>
-      <c r="M216" s="26"/>
-      <c r="N216" s="26"/>
-      <c r="O216" s="26"/>
-      <c r="P216" s="26"/>
-      <c r="Q216" s="26"/>
-      <c r="R216" s="26"/>
-      <c r="S216" s="26"/>
+      <c r="L216" s="25"/>
+      <c r="M216" s="25"/>
+      <c r="N216" s="25"/>
+      <c r="O216" s="25"/>
+      <c r="P216" s="25"/>
+      <c r="Q216" s="25"/>
+      <c r="R216" s="25"/>
+      <c r="S216" s="25"/>
     </row>
     <row r="217" spans="3:19" ht="12.75" x14ac:dyDescent="0.2">
       <c r="C217" s="21" t="s">
@@ -7950,14 +7991,14 @@
       <c r="J230" s="17">
         <v>1738648.8324483824</v>
       </c>
-      <c r="L230" s="26"/>
-      <c r="M230" s="26"/>
-      <c r="N230" s="26"/>
-      <c r="O230" s="26"/>
-      <c r="P230" s="26"/>
-      <c r="Q230" s="26"/>
-      <c r="R230" s="26"/>
-      <c r="S230" s="26"/>
+      <c r="L230" s="25"/>
+      <c r="M230" s="25"/>
+      <c r="N230" s="25"/>
+      <c r="O230" s="25"/>
+      <c r="P230" s="25"/>
+      <c r="Q230" s="25"/>
+      <c r="R230" s="25"/>
+      <c r="S230" s="25"/>
     </row>
     <row r="231" spans="3:19" ht="12.75" x14ac:dyDescent="0.2">
       <c r="C231" s="21" t="s">
@@ -8410,14 +8451,14 @@
       <c r="J244" s="17">
         <v>1985410.7822452041</v>
       </c>
-      <c r="L244" s="26"/>
-      <c r="M244" s="26"/>
-      <c r="N244" s="26"/>
-      <c r="O244" s="26"/>
-      <c r="P244" s="26"/>
-      <c r="Q244" s="26"/>
-      <c r="R244" s="26"/>
-      <c r="S244" s="26"/>
+      <c r="L244" s="25"/>
+      <c r="M244" s="25"/>
+      <c r="N244" s="25"/>
+      <c r="O244" s="25"/>
+      <c r="P244" s="25"/>
+      <c r="Q244" s="25"/>
+      <c r="R244" s="25"/>
+      <c r="S244" s="25"/>
     </row>
     <row r="245" spans="3:19" ht="12.75" x14ac:dyDescent="0.2">
       <c r="C245" s="21" t="s">
@@ -8870,14 +8911,14 @@
       <c r="J258" s="17">
         <v>2291605.1338285003</v>
       </c>
-      <c r="L258" s="26"/>
-      <c r="M258" s="26"/>
-      <c r="N258" s="26"/>
-      <c r="O258" s="26"/>
-      <c r="P258" s="26"/>
-      <c r="Q258" s="26"/>
-      <c r="R258" s="26"/>
-      <c r="S258" s="26"/>
+      <c r="L258" s="25"/>
+      <c r="M258" s="25"/>
+      <c r="N258" s="25"/>
+      <c r="O258" s="25"/>
+      <c r="P258" s="25"/>
+      <c r="Q258" s="25"/>
+      <c r="R258" s="25"/>
+      <c r="S258" s="25"/>
     </row>
     <row r="259" spans="3:19" ht="12.75" x14ac:dyDescent="0.2">
       <c r="C259" s="21" t="s">
@@ -9330,14 +9371,14 @@
       <c r="J272" s="17">
         <v>2414382.2767177997</v>
       </c>
-      <c r="L272" s="26"/>
-      <c r="M272" s="26"/>
-      <c r="N272" s="26"/>
-      <c r="O272" s="26"/>
-      <c r="P272" s="26"/>
-      <c r="Q272" s="26"/>
-      <c r="R272" s="26"/>
-      <c r="S272" s="26"/>
+      <c r="L272" s="25"/>
+      <c r="M272" s="25"/>
+      <c r="N272" s="25"/>
+      <c r="O272" s="25"/>
+      <c r="P272" s="25"/>
+      <c r="Q272" s="25"/>
+      <c r="R272" s="25"/>
+      <c r="S272" s="25"/>
     </row>
     <row r="273" spans="3:19" ht="12.75" x14ac:dyDescent="0.2">
       <c r="C273" s="21" t="s">
@@ -9790,14 +9831,14 @@
       <c r="J286" s="17">
         <v>2657649.54</v>
       </c>
-      <c r="L286" s="26"/>
-      <c r="M286" s="26"/>
-      <c r="N286" s="26"/>
-      <c r="O286" s="26"/>
-      <c r="P286" s="26"/>
-      <c r="Q286" s="26"/>
-      <c r="R286" s="26"/>
-      <c r="S286" s="26"/>
+      <c r="L286" s="25"/>
+      <c r="M286" s="25"/>
+      <c r="N286" s="25"/>
+      <c r="O286" s="25"/>
+      <c r="P286" s="25"/>
+      <c r="Q286" s="25"/>
+      <c r="R286" s="25"/>
+      <c r="S286" s="25"/>
     </row>
     <row r="287" spans="3:19" ht="12.75" x14ac:dyDescent="0.2">
       <c r="C287" s="21" t="s">
@@ -10250,14 +10291,14 @@
       <c r="J300" s="17">
         <v>2714089.1319999998</v>
       </c>
-      <c r="L300" s="26"/>
-      <c r="M300" s="26"/>
-      <c r="N300" s="26"/>
-      <c r="O300" s="26"/>
-      <c r="P300" s="26"/>
-      <c r="Q300" s="26"/>
-      <c r="R300" s="26"/>
-      <c r="S300" s="26"/>
+      <c r="L300" s="25"/>
+      <c r="M300" s="25"/>
+      <c r="N300" s="25"/>
+      <c r="O300" s="25"/>
+      <c r="P300" s="25"/>
+      <c r="Q300" s="25"/>
+      <c r="R300" s="25"/>
+      <c r="S300" s="25"/>
     </row>
     <row r="301" spans="3:19" ht="12.75" x14ac:dyDescent="0.2">
       <c r="C301" s="21" t="s">
@@ -10710,14 +10751,14 @@
       <c r="J314" s="17">
         <v>3061147.3109999998</v>
       </c>
-      <c r="L314" s="26"/>
-      <c r="M314" s="26"/>
-      <c r="N314" s="26"/>
-      <c r="O314" s="26"/>
-      <c r="P314" s="26"/>
-      <c r="Q314" s="26"/>
-      <c r="R314" s="26"/>
-      <c r="S314" s="26"/>
+      <c r="L314" s="25"/>
+      <c r="M314" s="25"/>
+      <c r="N314" s="25"/>
+      <c r="O314" s="25"/>
+      <c r="P314" s="25"/>
+      <c r="Q314" s="25"/>
+      <c r="R314" s="25"/>
+      <c r="S314" s="25"/>
     </row>
     <row r="315" spans="3:19" ht="12.75" x14ac:dyDescent="0.2">
       <c r="C315" s="21" t="s">
@@ -11170,14 +11211,14 @@
       <c r="J328" s="17">
         <v>3336939.5144332</v>
       </c>
-      <c r="L328" s="26"/>
-      <c r="M328" s="26"/>
-      <c r="N328" s="26"/>
-      <c r="O328" s="26"/>
-      <c r="P328" s="26"/>
-      <c r="Q328" s="26"/>
-      <c r="R328" s="26"/>
-      <c r="S328" s="26"/>
+      <c r="L328" s="25"/>
+      <c r="M328" s="25"/>
+      <c r="N328" s="25"/>
+      <c r="O328" s="25"/>
+      <c r="P328" s="25"/>
+      <c r="Q328" s="25"/>
+      <c r="R328" s="25"/>
+      <c r="S328" s="25"/>
     </row>
     <row r="329" spans="3:19" ht="12.75" x14ac:dyDescent="0.2">
       <c r="C329" s="21" t="s">
@@ -11630,14 +11671,14 @@
       <c r="J342" s="17">
         <v>3468208.7130000005</v>
       </c>
-      <c r="L342" s="26"/>
-      <c r="M342" s="26"/>
-      <c r="N342" s="26"/>
-      <c r="O342" s="26"/>
-      <c r="P342" s="26"/>
-      <c r="Q342" s="26"/>
-      <c r="R342" s="26"/>
-      <c r="S342" s="26"/>
+      <c r="L342" s="25"/>
+      <c r="M342" s="25"/>
+      <c r="N342" s="25"/>
+      <c r="O342" s="25"/>
+      <c r="P342" s="25"/>
+      <c r="Q342" s="25"/>
+      <c r="R342" s="25"/>
+      <c r="S342" s="25"/>
     </row>
     <row r="343" spans="3:19" ht="12.75" x14ac:dyDescent="0.2">
       <c r="C343" s="21" t="s">
@@ -12090,14 +12131,14 @@
       <c r="J356" s="17">
         <v>3601337.2899999996</v>
       </c>
-      <c r="L356" s="26"/>
-      <c r="M356" s="26"/>
-      <c r="N356" s="26"/>
-      <c r="O356" s="26"/>
-      <c r="P356" s="26"/>
-      <c r="Q356" s="26"/>
-      <c r="R356" s="26"/>
-      <c r="S356" s="26"/>
+      <c r="L356" s="25"/>
+      <c r="M356" s="25"/>
+      <c r="N356" s="25"/>
+      <c r="O356" s="25"/>
+      <c r="P356" s="25"/>
+      <c r="Q356" s="25"/>
+      <c r="R356" s="25"/>
+      <c r="S356" s="25"/>
     </row>
     <row r="357" spans="3:19" ht="12.75" x14ac:dyDescent="0.2">
       <c r="C357" s="21" t="s">
@@ -12550,14 +12591,14 @@
       <c r="J370" s="17">
         <v>3610988.6924000001</v>
       </c>
-      <c r="L370" s="26"/>
-      <c r="M370" s="26"/>
-      <c r="N370" s="26"/>
-      <c r="O370" s="26"/>
-      <c r="P370" s="26"/>
-      <c r="Q370" s="26"/>
-      <c r="R370" s="26"/>
-      <c r="S370" s="26"/>
+      <c r="L370" s="25"/>
+      <c r="M370" s="25"/>
+      <c r="N370" s="25"/>
+      <c r="O370" s="25"/>
+      <c r="P370" s="25"/>
+      <c r="Q370" s="25"/>
+      <c r="R370" s="25"/>
+      <c r="S370" s="25"/>
     </row>
     <row r="371" spans="3:19" ht="12.75" x14ac:dyDescent="0.2">
       <c r="C371" s="21" t="s">
@@ -13010,14 +13051,14 @@
       <c r="J384" s="17">
         <v>3757392.0140000004</v>
       </c>
-      <c r="L384" s="26"/>
-      <c r="M384" s="26"/>
-      <c r="N384" s="26"/>
-      <c r="O384" s="26"/>
-      <c r="P384" s="26"/>
-      <c r="Q384" s="26"/>
-      <c r="R384" s="26"/>
-      <c r="S384" s="26"/>
+      <c r="L384" s="25"/>
+      <c r="M384" s="25"/>
+      <c r="N384" s="25"/>
+      <c r="O384" s="25"/>
+      <c r="P384" s="25"/>
+      <c r="Q384" s="25"/>
+      <c r="R384" s="25"/>
+      <c r="S384" s="25"/>
     </row>
     <row r="385" spans="3:19" ht="12.75" x14ac:dyDescent="0.2">
       <c r="C385" s="21" t="s">
@@ -13470,14 +13511,14 @@
       <c r="J398" s="17">
         <v>3900345.2380000004</v>
       </c>
-      <c r="L398" s="26"/>
-      <c r="M398" s="26"/>
-      <c r="N398" s="26"/>
-      <c r="O398" s="26"/>
-      <c r="P398" s="26"/>
-      <c r="Q398" s="26"/>
-      <c r="R398" s="26"/>
-      <c r="S398" s="26"/>
+      <c r="L398" s="25"/>
+      <c r="M398" s="25"/>
+      <c r="N398" s="25"/>
+      <c r="O398" s="25"/>
+      <c r="P398" s="25"/>
+      <c r="Q398" s="25"/>
+      <c r="R398" s="25"/>
+      <c r="S398" s="25"/>
     </row>
     <row r="399" spans="3:19" ht="12.75" x14ac:dyDescent="0.2">
       <c r="C399" s="21" t="s">
@@ -13931,14 +13972,14 @@
         <v>3206833.645</v>
       </c>
       <c r="K412" s="7"/>
-      <c r="L412" s="26"/>
-      <c r="M412" s="26"/>
-      <c r="N412" s="26"/>
-      <c r="O412" s="26"/>
-      <c r="P412" s="26"/>
-      <c r="Q412" s="26"/>
-      <c r="R412" s="26"/>
-      <c r="S412" s="26"/>
+      <c r="L412" s="25"/>
+      <c r="M412" s="25"/>
+      <c r="N412" s="25"/>
+      <c r="O412" s="25"/>
+      <c r="P412" s="25"/>
+      <c r="Q412" s="25"/>
+      <c r="R412" s="25"/>
+      <c r="S412" s="25"/>
     </row>
     <row r="413" spans="3:19" ht="12.75" x14ac:dyDescent="0.2">
       <c r="C413" s="21" t="s">
@@ -14401,14 +14442,14 @@
         <v>3606958.7226859862</v>
       </c>
       <c r="K426" s="6"/>
-      <c r="L426" s="26"/>
-      <c r="M426" s="26"/>
-      <c r="N426" s="26"/>
-      <c r="O426" s="26"/>
-      <c r="P426" s="26"/>
-      <c r="Q426" s="26"/>
-      <c r="R426" s="26"/>
-      <c r="S426" s="26"/>
+      <c r="L426" s="25"/>
+      <c r="M426" s="25"/>
+      <c r="N426" s="25"/>
+      <c r="O426" s="25"/>
+      <c r="P426" s="25"/>
+      <c r="Q426" s="25"/>
+      <c r="R426" s="25"/>
+      <c r="S426" s="25"/>
     </row>
     <row r="427" spans="3:19" ht="12.75" x14ac:dyDescent="0.2">
       <c r="C427" s="21" t="s">
@@ -14875,14 +14916,14 @@
         <v>3888570.9300095243</v>
       </c>
       <c r="K440" s="6"/>
-      <c r="L440" s="26"/>
-      <c r="M440" s="26"/>
-      <c r="N440" s="26"/>
-      <c r="O440" s="26"/>
-      <c r="P440" s="26"/>
-      <c r="Q440" s="26"/>
-      <c r="R440" s="26"/>
-      <c r="S440" s="26"/>
+      <c r="L440" s="25"/>
+      <c r="M440" s="25"/>
+      <c r="N440" s="25"/>
+      <c r="O440" s="25"/>
+      <c r="P440" s="25"/>
+      <c r="Q440" s="25"/>
+      <c r="R440" s="25"/>
+      <c r="S440" s="25"/>
     </row>
     <row r="441" spans="3:19" ht="12.75" x14ac:dyDescent="0.2">
       <c r="C441" s="21" t="s">
@@ -15349,14 +15390,14 @@
         <v>3977360.585</v>
       </c>
       <c r="K454" s="6"/>
-      <c r="L454" s="26"/>
-      <c r="M454" s="26"/>
-      <c r="N454" s="26"/>
-      <c r="O454" s="26"/>
-      <c r="P454" s="26"/>
-      <c r="Q454" s="26"/>
-      <c r="R454" s="26"/>
-      <c r="S454" s="26"/>
+      <c r="L454" s="25"/>
+      <c r="M454" s="25"/>
+      <c r="N454" s="25"/>
+      <c r="O454" s="25"/>
+      <c r="P454" s="25"/>
+      <c r="Q454" s="25"/>
+      <c r="R454" s="25"/>
+      <c r="S454" s="25"/>
     </row>
     <row r="455" spans="3:19" ht="12.75" x14ac:dyDescent="0.2">
       <c r="C455" s="21" t="s">
@@ -16747,28 +16788,28 @@
     </row>
     <row r="496" spans="3:19" ht="13.5" x14ac:dyDescent="0.2">
       <c r="C496" s="20" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D496" s="24">
-        <v>170467.84999999998</v>
+        <v>232507.33999999997</v>
       </c>
       <c r="E496" s="24">
-        <v>184012.51</v>
+        <v>239755.66000000003</v>
       </c>
       <c r="F496" s="24">
-        <v>114275</v>
+        <v>152769</v>
       </c>
       <c r="G496" s="24">
-        <v>46391.58</v>
+        <v>76857.11</v>
       </c>
       <c r="H496" s="24">
-        <v>34045.840000000004</v>
+        <v>46423.880000000005</v>
       </c>
       <c r="I496" s="24">
-        <v>248630.05900000001</v>
+        <v>310400.86800000002</v>
       </c>
       <c r="J496" s="24">
-        <v>797822.83900000004</v>
+        <v>1058713.858</v>
       </c>
       <c r="K496" s="6"/>
       <c r="L496" s="3"/>
@@ -16784,25 +16825,25 @@
       <c r="C497" s="21" t="s">
         <v>0</v>
       </c>
-      <c r="D497" s="28">
+      <c r="D497" s="27">
         <v>59030.229999999996</v>
       </c>
-      <c r="E497" s="28">
+      <c r="E497" s="27">
         <v>94628.85</v>
       </c>
-      <c r="F497" s="28">
+      <c r="F497" s="27">
         <v>50403</v>
       </c>
-      <c r="G497" s="28">
+      <c r="G497" s="27">
         <v>8424</v>
       </c>
-      <c r="H497" s="28">
+      <c r="H497" s="27">
         <v>13745.490000000002</v>
       </c>
-      <c r="I497" s="28">
+      <c r="I497" s="27">
         <v>103548.052</v>
       </c>
-      <c r="J497" s="28">
+      <c r="J497" s="27">
         <v>329779.62199999997</v>
       </c>
       <c r="K497" s="6"/>
@@ -16819,25 +16860,25 @@
       <c r="C498" s="21" t="s">
         <v>1</v>
       </c>
-      <c r="D498" s="28">
+      <c r="D498" s="27">
         <v>49961.399999999994</v>
       </c>
-      <c r="E498" s="28">
+      <c r="E498" s="27">
         <v>37817.950000000004</v>
       </c>
-      <c r="F498" s="28">
+      <c r="F498" s="27">
         <v>27094</v>
       </c>
-      <c r="G498" s="28">
+      <c r="G498" s="27">
         <v>14712.72</v>
       </c>
-      <c r="H498" s="28">
+      <c r="H498" s="27">
         <v>10184.650000000001</v>
       </c>
-      <c r="I498" s="28">
+      <c r="I498" s="27">
         <v>68268.429999999993</v>
       </c>
-      <c r="J498" s="28">
+      <c r="J498" s="27">
         <v>208039.15</v>
       </c>
       <c r="K498" s="6"/>
@@ -16854,25 +16895,25 @@
       <c r="C499" s="21" t="s">
         <v>2</v>
       </c>
-      <c r="D499" s="28">
+      <c r="D499" s="27">
         <v>61476.22</v>
       </c>
-      <c r="E499" s="28">
+      <c r="E499" s="27">
         <v>51565.710000000006</v>
       </c>
-      <c r="F499" s="28">
+      <c r="F499" s="27">
         <v>36778</v>
       </c>
-      <c r="G499" s="28">
+      <c r="G499" s="27">
         <v>23254.86</v>
       </c>
-      <c r="H499" s="28">
+      <c r="H499" s="27">
         <v>10115.700000000001</v>
       </c>
-      <c r="I499" s="28">
+      <c r="I499" s="27">
         <v>76813.577000000005</v>
       </c>
-      <c r="J499" s="28">
+      <c r="J499" s="27">
         <v>260004.06699999998</v>
       </c>
       <c r="K499" s="6"/>
@@ -16886,14 +16927,30 @@
       <c r="S499" s="3"/>
     </row>
     <row r="500" spans="3:19" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="C500" s="22"/>
-      <c r="D500" s="25"/>
-      <c r="E500" s="25"/>
-      <c r="F500" s="25"/>
-      <c r="G500" s="25"/>
-      <c r="H500" s="25"/>
-      <c r="I500" s="25"/>
-      <c r="J500" s="25"/>
+      <c r="C500" s="22" t="s">
+        <v>3</v>
+      </c>
+      <c r="D500" s="29">
+        <v>62039.49</v>
+      </c>
+      <c r="E500" s="29">
+        <v>55743.150000000009</v>
+      </c>
+      <c r="F500" s="29">
+        <v>38494</v>
+      </c>
+      <c r="G500" s="29">
+        <v>30465.53</v>
+      </c>
+      <c r="H500" s="29">
+        <v>12378.039999999999</v>
+      </c>
+      <c r="I500" s="29">
+        <v>61770.809000000001</v>
+      </c>
+      <c r="J500" s="29">
+        <v>260891.01900000003</v>
+      </c>
       <c r="K500" s="6"/>
       <c r="L500" s="3"/>
       <c r="M500" s="3"/>
@@ -16905,8 +16962,8 @@
       <c r="S500" s="3"/>
     </row>
     <row r="501" spans="3:19" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="C501" s="9" t="s">
-        <v>24</v>
+      <c r="C501" s="28" t="s">
+        <v>23</v>
       </c>
       <c r="D501" s="2"/>
       <c r="E501" s="2"/>
@@ -16916,20 +16973,20 @@
       <c r="J501" s="2"/>
     </row>
     <row r="502" spans="3:19" x14ac:dyDescent="0.2">
-      <c r="C502" s="9" t="s">
-        <v>23</v>
+      <c r="C502" s="28" t="s">
+        <v>26</v>
       </c>
       <c r="I502" s="4"/>
     </row>
     <row r="503" spans="3:19" x14ac:dyDescent="0.2">
       <c r="C503" s="9"/>
-      <c r="D503" s="27"/>
-      <c r="E503" s="27"/>
-      <c r="F503" s="27"/>
-      <c r="G503" s="27"/>
-      <c r="H503" s="27"/>
-      <c r="I503" s="27"/>
-      <c r="J503" s="27"/>
+      <c r="D503" s="26"/>
+      <c r="E503" s="26"/>
+      <c r="F503" s="26"/>
+      <c r="G503" s="26"/>
+      <c r="H503" s="26"/>
+      <c r="I503" s="26"/>
+      <c r="J503" s="26"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
auto: actualizar indicadores adelantados 2026-08-17
</commit_message>
<xml_diff>
--- a/datos/indicadores_adelantados/cemento/produccion_cemento_depto_1991_2026.xlsx
+++ b/datos/indicadores_adelantados/cemento/produccion_cemento_depto_1991_2026.xlsx
@@ -1,16 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="24332"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="5" rupBuild="14420"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="U:\1. Página Web\2026 - 06. Junio\Cemento 04-2026\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="Z:\3. IGAE\2026-08 Agosto\5. Cemento\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FF863199-B5E4-425C-A30C-26E066413708}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="270" windowWidth="25440" windowHeight="15270" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="10440" windowHeight="11010"/>
   </bookViews>
   <sheets>
     <sheet name="C1" sheetId="1" r:id="rId1"/>
@@ -25,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="439" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="439" uniqueCount="26">
   <si>
     <t>Enero</t>
   </si>
@@ -91,11 +90,10 @@
   </si>
   <si>
     <r>
-      <t>2024</t>
+      <t xml:space="preserve">             </t>
     </r>
     <r>
       <rPr>
-        <b/>
         <vertAlign val="superscript"/>
         <sz val="9"/>
         <rFont val="Arial"/>
@@ -103,20 +101,13 @@
       </rPr>
       <t>(p)</t>
     </r>
-  </si>
-  <si>
-    <r>
-      <t>2025</t>
-    </r>
     <r>
       <rPr>
-        <b/>
-        <vertAlign val="superscript"/>
         <sz val="9"/>
         <rFont val="Arial"/>
         <family val="2"/>
       </rPr>
-      <t>(p)</t>
+      <t xml:space="preserve"> : Preliminar</t>
     </r>
   </si>
   <si>
@@ -141,37 +132,18 @@
     <t>BOLIVIA: PRODUCCIÓN DE CEMENTO POR DEPARTAMENTO SEGÚN AÑO Y MES, 1991 - 2026</t>
   </si>
   <si>
-    <r>
-      <t xml:space="preserve">             </t>
-    </r>
-    <r>
-      <rPr>
-        <vertAlign val="superscript"/>
-        <sz val="8"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>(p)</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> : Preliminar</t>
-    </r>
+    <t xml:space="preserve">Mayo </t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <numFmts count="2">
     <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="164" formatCode="#,##0.00000"/>
   </numFmts>
-  <fonts count="16" x14ac:knownFonts="1">
+  <fonts count="15" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -263,13 +235,8 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="8"/>
-      <name val="Arial"/>
-      <family val="2"/>
-    </font>
-    <font>
       <vertAlign val="superscript"/>
-      <sz val="8"/>
+      <sz val="9"/>
       <name val="Arial"/>
       <family val="2"/>
     </font>
@@ -402,7 +369,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="13" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -466,15 +433,14 @@
     <xf numFmtId="3" fontId="7" fillId="5" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="3" fontId="8" fillId="3" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
     <xf numFmtId="43" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="3" fontId="8" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="3" fontId="8" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
   </cellXfs>
@@ -615,23 +581,6 @@
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri" panose="020F0502020204030204"/>
@@ -667,23 +616,6 @@
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -859,8 +791,8 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="C1:S503"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="C1:S506"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="2" width="1.42578125" style="2" customWidth="1"/>
@@ -1380,7 +1312,7 @@
     <row r="1" spans="3:19" ht="75.75" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="2" spans="3:19" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C2" s="12" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D2" s="12"/>
       <c r="E2" s="12"/>
@@ -1463,14 +1395,14 @@
       <c r="J6" s="17">
         <v>587056.95000000007</v>
       </c>
-      <c r="L6" s="25"/>
-      <c r="M6" s="25"/>
-      <c r="N6" s="25"/>
-      <c r="O6" s="25"/>
-      <c r="P6" s="25"/>
-      <c r="Q6" s="25"/>
-      <c r="R6" s="25"/>
-      <c r="S6" s="25"/>
+      <c r="L6" s="26"/>
+      <c r="M6" s="26"/>
+      <c r="N6" s="26"/>
+      <c r="O6" s="26"/>
+      <c r="P6" s="26"/>
+      <c r="Q6" s="26"/>
+      <c r="R6" s="26"/>
+      <c r="S6" s="26"/>
     </row>
     <row r="7" spans="3:19" s="3" customFormat="1" ht="12.75" x14ac:dyDescent="0.2">
       <c r="C7" s="21" t="s">
@@ -1819,14 +1751,14 @@
       <c r="J20" s="17">
         <v>649643.79</v>
       </c>
-      <c r="L20" s="25"/>
-      <c r="M20" s="25"/>
-      <c r="N20" s="25"/>
-      <c r="O20" s="25"/>
-      <c r="P20" s="25"/>
-      <c r="Q20" s="25"/>
-      <c r="R20" s="25"/>
-      <c r="S20" s="25"/>
+      <c r="L20" s="26"/>
+      <c r="M20" s="26"/>
+      <c r="N20" s="26"/>
+      <c r="O20" s="26"/>
+      <c r="P20" s="26"/>
+      <c r="Q20" s="26"/>
+      <c r="R20" s="26"/>
+      <c r="S20" s="26"/>
     </row>
     <row r="21" spans="3:19" s="3" customFormat="1" ht="12.75" x14ac:dyDescent="0.2">
       <c r="C21" s="21" t="s">
@@ -2175,14 +2107,14 @@
       <c r="J34" s="17">
         <v>717607.41</v>
       </c>
-      <c r="L34" s="25"/>
-      <c r="M34" s="25"/>
-      <c r="N34" s="25"/>
-      <c r="O34" s="25"/>
-      <c r="P34" s="25"/>
-      <c r="Q34" s="25"/>
-      <c r="R34" s="25"/>
-      <c r="S34" s="25"/>
+      <c r="L34" s="26"/>
+      <c r="M34" s="26"/>
+      <c r="N34" s="26"/>
+      <c r="O34" s="26"/>
+      <c r="P34" s="26"/>
+      <c r="Q34" s="26"/>
+      <c r="R34" s="26"/>
+      <c r="S34" s="26"/>
     </row>
     <row r="35" spans="3:19" s="3" customFormat="1" ht="12.75" x14ac:dyDescent="0.2">
       <c r="C35" s="21" t="s">
@@ -2531,14 +2463,14 @@
       <c r="J48" s="17">
         <v>776301.62999999989</v>
       </c>
-      <c r="L48" s="25"/>
-      <c r="M48" s="25"/>
-      <c r="N48" s="25"/>
-      <c r="O48" s="25"/>
-      <c r="P48" s="25"/>
-      <c r="Q48" s="25"/>
-      <c r="R48" s="25"/>
-      <c r="S48" s="25"/>
+      <c r="L48" s="26"/>
+      <c r="M48" s="26"/>
+      <c r="N48" s="26"/>
+      <c r="O48" s="26"/>
+      <c r="P48" s="26"/>
+      <c r="Q48" s="26"/>
+      <c r="R48" s="26"/>
+      <c r="S48" s="26"/>
     </row>
     <row r="49" spans="3:19" s="3" customFormat="1" ht="12.75" x14ac:dyDescent="0.2">
       <c r="C49" s="21" t="s">
@@ -2887,14 +2819,14 @@
       <c r="J62" s="17">
         <v>892430.95000000007</v>
       </c>
-      <c r="L62" s="25"/>
-      <c r="M62" s="25"/>
-      <c r="N62" s="25"/>
-      <c r="O62" s="25"/>
-      <c r="P62" s="25"/>
-      <c r="Q62" s="25"/>
-      <c r="R62" s="25"/>
-      <c r="S62" s="25"/>
+      <c r="L62" s="26"/>
+      <c r="M62" s="26"/>
+      <c r="N62" s="26"/>
+      <c r="O62" s="26"/>
+      <c r="P62" s="26"/>
+      <c r="Q62" s="26"/>
+      <c r="R62" s="26"/>
+      <c r="S62" s="26"/>
     </row>
     <row r="63" spans="3:19" s="3" customFormat="1" ht="12.75" x14ac:dyDescent="0.2">
       <c r="C63" s="21" t="s">
@@ -3243,14 +3175,14 @@
       <c r="J76" s="17">
         <v>900956.8</v>
       </c>
-      <c r="L76" s="25"/>
-      <c r="M76" s="25"/>
-      <c r="N76" s="25"/>
-      <c r="O76" s="25"/>
-      <c r="P76" s="25"/>
-      <c r="Q76" s="25"/>
-      <c r="R76" s="25"/>
-      <c r="S76" s="25"/>
+      <c r="L76" s="26"/>
+      <c r="M76" s="26"/>
+      <c r="N76" s="26"/>
+      <c r="O76" s="26"/>
+      <c r="P76" s="26"/>
+      <c r="Q76" s="26"/>
+      <c r="R76" s="26"/>
+      <c r="S76" s="26"/>
     </row>
     <row r="77" spans="3:19" s="3" customFormat="1" ht="12.75" x14ac:dyDescent="0.2">
       <c r="C77" s="21" t="s">
@@ -3599,14 +3531,14 @@
       <c r="J90" s="17">
         <v>1047951.0700000001</v>
       </c>
-      <c r="L90" s="25"/>
-      <c r="M90" s="25"/>
-      <c r="N90" s="25"/>
-      <c r="O90" s="25"/>
-      <c r="P90" s="25"/>
-      <c r="Q90" s="25"/>
-      <c r="R90" s="25"/>
-      <c r="S90" s="25"/>
+      <c r="L90" s="26"/>
+      <c r="M90" s="26"/>
+      <c r="N90" s="26"/>
+      <c r="O90" s="26"/>
+      <c r="P90" s="26"/>
+      <c r="Q90" s="26"/>
+      <c r="R90" s="26"/>
+      <c r="S90" s="26"/>
     </row>
     <row r="91" spans="3:19" s="3" customFormat="1" ht="12.75" x14ac:dyDescent="0.2">
       <c r="C91" s="21" t="s">
@@ -3955,14 +3887,14 @@
       <c r="J104" s="17">
         <v>1166511.1599999997</v>
       </c>
-      <c r="L104" s="25"/>
-      <c r="M104" s="25"/>
-      <c r="N104" s="25"/>
-      <c r="O104" s="25"/>
-      <c r="P104" s="25"/>
-      <c r="Q104" s="25"/>
-      <c r="R104" s="25"/>
-      <c r="S104" s="25"/>
+      <c r="L104" s="26"/>
+      <c r="M104" s="26"/>
+      <c r="N104" s="26"/>
+      <c r="O104" s="26"/>
+      <c r="P104" s="26"/>
+      <c r="Q104" s="26"/>
+      <c r="R104" s="26"/>
+      <c r="S104" s="26"/>
     </row>
     <row r="105" spans="3:19" s="3" customFormat="1" ht="12.75" x14ac:dyDescent="0.2">
       <c r="C105" s="21" t="s">
@@ -4311,14 +4243,14 @@
       <c r="J118" s="17">
         <v>1201274.32</v>
       </c>
-      <c r="L118" s="25"/>
-      <c r="M118" s="25"/>
-      <c r="N118" s="25"/>
-      <c r="O118" s="25"/>
-      <c r="P118" s="25"/>
-      <c r="Q118" s="25"/>
-      <c r="R118" s="25"/>
-      <c r="S118" s="25"/>
+      <c r="L118" s="26"/>
+      <c r="M118" s="26"/>
+      <c r="N118" s="26"/>
+      <c r="O118" s="26"/>
+      <c r="P118" s="26"/>
+      <c r="Q118" s="26"/>
+      <c r="R118" s="26"/>
+      <c r="S118" s="26"/>
     </row>
     <row r="119" spans="3:19" ht="12.75" x14ac:dyDescent="0.2">
       <c r="C119" s="21" t="s">
@@ -4771,14 +4703,14 @@
       <c r="J132" s="17">
         <v>1071941</v>
       </c>
-      <c r="L132" s="25"/>
-      <c r="M132" s="25"/>
-      <c r="N132" s="25"/>
-      <c r="O132" s="25"/>
-      <c r="P132" s="25"/>
-      <c r="Q132" s="25"/>
-      <c r="R132" s="25"/>
-      <c r="S132" s="25"/>
+      <c r="L132" s="26"/>
+      <c r="M132" s="26"/>
+      <c r="N132" s="26"/>
+      <c r="O132" s="26"/>
+      <c r="P132" s="26"/>
+      <c r="Q132" s="26"/>
+      <c r="R132" s="26"/>
+      <c r="S132" s="26"/>
     </row>
     <row r="133" spans="3:19" ht="12.75" x14ac:dyDescent="0.2">
       <c r="C133" s="21" t="s">
@@ -5231,14 +5163,14 @@
       <c r="J146" s="17">
         <v>982543.11</v>
       </c>
-      <c r="L146" s="25"/>
-      <c r="M146" s="25"/>
-      <c r="N146" s="25"/>
-      <c r="O146" s="25"/>
-      <c r="P146" s="25"/>
-      <c r="Q146" s="25"/>
-      <c r="R146" s="25"/>
-      <c r="S146" s="25"/>
+      <c r="L146" s="26"/>
+      <c r="M146" s="26"/>
+      <c r="N146" s="26"/>
+      <c r="O146" s="26"/>
+      <c r="P146" s="26"/>
+      <c r="Q146" s="26"/>
+      <c r="R146" s="26"/>
+      <c r="S146" s="26"/>
     </row>
     <row r="147" spans="3:19" ht="12.75" x14ac:dyDescent="0.2">
       <c r="C147" s="21" t="s">
@@ -5691,14 +5623,14 @@
       <c r="J160" s="17">
         <v>1010445.99</v>
       </c>
-      <c r="L160" s="25"/>
-      <c r="M160" s="25"/>
-      <c r="N160" s="25"/>
-      <c r="O160" s="25"/>
-      <c r="P160" s="25"/>
-      <c r="Q160" s="25"/>
-      <c r="R160" s="25"/>
-      <c r="S160" s="25"/>
+      <c r="L160" s="26"/>
+      <c r="M160" s="26"/>
+      <c r="N160" s="26"/>
+      <c r="O160" s="26"/>
+      <c r="P160" s="26"/>
+      <c r="Q160" s="26"/>
+      <c r="R160" s="26"/>
+      <c r="S160" s="26"/>
     </row>
     <row r="161" spans="3:19" ht="12.75" x14ac:dyDescent="0.2">
       <c r="C161" s="21" t="s">
@@ -6151,14 +6083,14 @@
       <c r="J174" s="17">
         <v>1138146.21</v>
       </c>
-      <c r="L174" s="25"/>
-      <c r="M174" s="25"/>
-      <c r="N174" s="25"/>
-      <c r="O174" s="25"/>
-      <c r="P174" s="25"/>
-      <c r="Q174" s="25"/>
-      <c r="R174" s="25"/>
-      <c r="S174" s="25"/>
+      <c r="L174" s="26"/>
+      <c r="M174" s="26"/>
+      <c r="N174" s="26"/>
+      <c r="O174" s="26"/>
+      <c r="P174" s="26"/>
+      <c r="Q174" s="26"/>
+      <c r="R174" s="26"/>
+      <c r="S174" s="26"/>
     </row>
     <row r="175" spans="3:19" ht="12.75" x14ac:dyDescent="0.2">
       <c r="C175" s="21" t="s">
@@ -6611,14 +6543,14 @@
       <c r="J188" s="17">
         <v>1276411.5103322999</v>
       </c>
-      <c r="L188" s="25"/>
-      <c r="M188" s="25"/>
-      <c r="N188" s="25"/>
-      <c r="O188" s="25"/>
-      <c r="P188" s="25"/>
-      <c r="Q188" s="25"/>
-      <c r="R188" s="25"/>
-      <c r="S188" s="25"/>
+      <c r="L188" s="26"/>
+      <c r="M188" s="26"/>
+      <c r="N188" s="26"/>
+      <c r="O188" s="26"/>
+      <c r="P188" s="26"/>
+      <c r="Q188" s="26"/>
+      <c r="R188" s="26"/>
+      <c r="S188" s="26"/>
     </row>
     <row r="189" spans="3:19" ht="12.75" x14ac:dyDescent="0.2">
       <c r="C189" s="21" t="s">
@@ -7071,14 +7003,14 @@
       <c r="J202" s="17">
         <v>1439951.1600000001</v>
       </c>
-      <c r="L202" s="25"/>
-      <c r="M202" s="25"/>
-      <c r="N202" s="25"/>
-      <c r="O202" s="25"/>
-      <c r="P202" s="25"/>
-      <c r="Q202" s="25"/>
-      <c r="R202" s="25"/>
-      <c r="S202" s="25"/>
+      <c r="L202" s="26"/>
+      <c r="M202" s="26"/>
+      <c r="N202" s="26"/>
+      <c r="O202" s="26"/>
+      <c r="P202" s="26"/>
+      <c r="Q202" s="26"/>
+      <c r="R202" s="26"/>
+      <c r="S202" s="26"/>
     </row>
     <row r="203" spans="3:19" ht="12.75" x14ac:dyDescent="0.2">
       <c r="C203" s="21" t="s">
@@ -7531,14 +7463,14 @@
       <c r="J216" s="17">
         <v>1636078.7199999997</v>
       </c>
-      <c r="L216" s="25"/>
-      <c r="M216" s="25"/>
-      <c r="N216" s="25"/>
-      <c r="O216" s="25"/>
-      <c r="P216" s="25"/>
-      <c r="Q216" s="25"/>
-      <c r="R216" s="25"/>
-      <c r="S216" s="25"/>
+      <c r="L216" s="26"/>
+      <c r="M216" s="26"/>
+      <c r="N216" s="26"/>
+      <c r="O216" s="26"/>
+      <c r="P216" s="26"/>
+      <c r="Q216" s="26"/>
+      <c r="R216" s="26"/>
+      <c r="S216" s="26"/>
     </row>
     <row r="217" spans="3:19" ht="12.75" x14ac:dyDescent="0.2">
       <c r="C217" s="21" t="s">
@@ -7991,14 +7923,14 @@
       <c r="J230" s="17">
         <v>1738648.8324483824</v>
       </c>
-      <c r="L230" s="25"/>
-      <c r="M230" s="25"/>
-      <c r="N230" s="25"/>
-      <c r="O230" s="25"/>
-      <c r="P230" s="25"/>
-      <c r="Q230" s="25"/>
-      <c r="R230" s="25"/>
-      <c r="S230" s="25"/>
+      <c r="L230" s="26"/>
+      <c r="M230" s="26"/>
+      <c r="N230" s="26"/>
+      <c r="O230" s="26"/>
+      <c r="P230" s="26"/>
+      <c r="Q230" s="26"/>
+      <c r="R230" s="26"/>
+      <c r="S230" s="26"/>
     </row>
     <row r="231" spans="3:19" ht="12.75" x14ac:dyDescent="0.2">
       <c r="C231" s="21" t="s">
@@ -8451,14 +8383,14 @@
       <c r="J244" s="17">
         <v>1985410.7822452041</v>
       </c>
-      <c r="L244" s="25"/>
-      <c r="M244" s="25"/>
-      <c r="N244" s="25"/>
-      <c r="O244" s="25"/>
-      <c r="P244" s="25"/>
-      <c r="Q244" s="25"/>
-      <c r="R244" s="25"/>
-      <c r="S244" s="25"/>
+      <c r="L244" s="26"/>
+      <c r="M244" s="26"/>
+      <c r="N244" s="26"/>
+      <c r="O244" s="26"/>
+      <c r="P244" s="26"/>
+      <c r="Q244" s="26"/>
+      <c r="R244" s="26"/>
+      <c r="S244" s="26"/>
     </row>
     <row r="245" spans="3:19" ht="12.75" x14ac:dyDescent="0.2">
       <c r="C245" s="21" t="s">
@@ -8911,14 +8843,14 @@
       <c r="J258" s="17">
         <v>2291605.1338285003</v>
       </c>
-      <c r="L258" s="25"/>
-      <c r="M258" s="25"/>
-      <c r="N258" s="25"/>
-      <c r="O258" s="25"/>
-      <c r="P258" s="25"/>
-      <c r="Q258" s="25"/>
-      <c r="R258" s="25"/>
-      <c r="S258" s="25"/>
+      <c r="L258" s="26"/>
+      <c r="M258" s="26"/>
+      <c r="N258" s="26"/>
+      <c r="O258" s="26"/>
+      <c r="P258" s="26"/>
+      <c r="Q258" s="26"/>
+      <c r="R258" s="26"/>
+      <c r="S258" s="26"/>
     </row>
     <row r="259" spans="3:19" ht="12.75" x14ac:dyDescent="0.2">
       <c r="C259" s="21" t="s">
@@ -9371,14 +9303,14 @@
       <c r="J272" s="17">
         <v>2414382.2767177997</v>
       </c>
-      <c r="L272" s="25"/>
-      <c r="M272" s="25"/>
-      <c r="N272" s="25"/>
-      <c r="O272" s="25"/>
-      <c r="P272" s="25"/>
-      <c r="Q272" s="25"/>
-      <c r="R272" s="25"/>
-      <c r="S272" s="25"/>
+      <c r="L272" s="26"/>
+      <c r="M272" s="26"/>
+      <c r="N272" s="26"/>
+      <c r="O272" s="26"/>
+      <c r="P272" s="26"/>
+      <c r="Q272" s="26"/>
+      <c r="R272" s="26"/>
+      <c r="S272" s="26"/>
     </row>
     <row r="273" spans="3:19" ht="12.75" x14ac:dyDescent="0.2">
       <c r="C273" s="21" t="s">
@@ -9831,14 +9763,14 @@
       <c r="J286" s="17">
         <v>2657649.54</v>
       </c>
-      <c r="L286" s="25"/>
-      <c r="M286" s="25"/>
-      <c r="N286" s="25"/>
-      <c r="O286" s="25"/>
-      <c r="P286" s="25"/>
-      <c r="Q286" s="25"/>
-      <c r="R286" s="25"/>
-      <c r="S286" s="25"/>
+      <c r="L286" s="26"/>
+      <c r="M286" s="26"/>
+      <c r="N286" s="26"/>
+      <c r="O286" s="26"/>
+      <c r="P286" s="26"/>
+      <c r="Q286" s="26"/>
+      <c r="R286" s="26"/>
+      <c r="S286" s="26"/>
     </row>
     <row r="287" spans="3:19" ht="12.75" x14ac:dyDescent="0.2">
       <c r="C287" s="21" t="s">
@@ -10291,14 +10223,14 @@
       <c r="J300" s="17">
         <v>2714089.1319999998</v>
       </c>
-      <c r="L300" s="25"/>
-      <c r="M300" s="25"/>
-      <c r="N300" s="25"/>
-      <c r="O300" s="25"/>
-      <c r="P300" s="25"/>
-      <c r="Q300" s="25"/>
-      <c r="R300" s="25"/>
-      <c r="S300" s="25"/>
+      <c r="L300" s="26"/>
+      <c r="M300" s="26"/>
+      <c r="N300" s="26"/>
+      <c r="O300" s="26"/>
+      <c r="P300" s="26"/>
+      <c r="Q300" s="26"/>
+      <c r="R300" s="26"/>
+      <c r="S300" s="26"/>
     </row>
     <row r="301" spans="3:19" ht="12.75" x14ac:dyDescent="0.2">
       <c r="C301" s="21" t="s">
@@ -10751,14 +10683,14 @@
       <c r="J314" s="17">
         <v>3061147.3109999998</v>
       </c>
-      <c r="L314" s="25"/>
-      <c r="M314" s="25"/>
-      <c r="N314" s="25"/>
-      <c r="O314" s="25"/>
-      <c r="P314" s="25"/>
-      <c r="Q314" s="25"/>
-      <c r="R314" s="25"/>
-      <c r="S314" s="25"/>
+      <c r="L314" s="26"/>
+      <c r="M314" s="26"/>
+      <c r="N314" s="26"/>
+      <c r="O314" s="26"/>
+      <c r="P314" s="26"/>
+      <c r="Q314" s="26"/>
+      <c r="R314" s="26"/>
+      <c r="S314" s="26"/>
     </row>
     <row r="315" spans="3:19" ht="12.75" x14ac:dyDescent="0.2">
       <c r="C315" s="21" t="s">
@@ -11211,14 +11143,14 @@
       <c r="J328" s="17">
         <v>3336939.5144332</v>
       </c>
-      <c r="L328" s="25"/>
-      <c r="M328" s="25"/>
-      <c r="N328" s="25"/>
-      <c r="O328" s="25"/>
-      <c r="P328" s="25"/>
-      <c r="Q328" s="25"/>
-      <c r="R328" s="25"/>
-      <c r="S328" s="25"/>
+      <c r="L328" s="26"/>
+      <c r="M328" s="26"/>
+      <c r="N328" s="26"/>
+      <c r="O328" s="26"/>
+      <c r="P328" s="26"/>
+      <c r="Q328" s="26"/>
+      <c r="R328" s="26"/>
+      <c r="S328" s="26"/>
     </row>
     <row r="329" spans="3:19" ht="12.75" x14ac:dyDescent="0.2">
       <c r="C329" s="21" t="s">
@@ -11671,14 +11603,14 @@
       <c r="J342" s="17">
         <v>3468208.7130000005</v>
       </c>
-      <c r="L342" s="25"/>
-      <c r="M342" s="25"/>
-      <c r="N342" s="25"/>
-      <c r="O342" s="25"/>
-      <c r="P342" s="25"/>
-      <c r="Q342" s="25"/>
-      <c r="R342" s="25"/>
-      <c r="S342" s="25"/>
+      <c r="L342" s="26"/>
+      <c r="M342" s="26"/>
+      <c r="N342" s="26"/>
+      <c r="O342" s="26"/>
+      <c r="P342" s="26"/>
+      <c r="Q342" s="26"/>
+      <c r="R342" s="26"/>
+      <c r="S342" s="26"/>
     </row>
     <row r="343" spans="3:19" ht="12.75" x14ac:dyDescent="0.2">
       <c r="C343" s="21" t="s">
@@ -12131,14 +12063,14 @@
       <c r="J356" s="17">
         <v>3601337.2899999996</v>
       </c>
-      <c r="L356" s="25"/>
-      <c r="M356" s="25"/>
-      <c r="N356" s="25"/>
-      <c r="O356" s="25"/>
-      <c r="P356" s="25"/>
-      <c r="Q356" s="25"/>
-      <c r="R356" s="25"/>
-      <c r="S356" s="25"/>
+      <c r="L356" s="26"/>
+      <c r="M356" s="26"/>
+      <c r="N356" s="26"/>
+      <c r="O356" s="26"/>
+      <c r="P356" s="26"/>
+      <c r="Q356" s="26"/>
+      <c r="R356" s="26"/>
+      <c r="S356" s="26"/>
     </row>
     <row r="357" spans="3:19" ht="12.75" x14ac:dyDescent="0.2">
       <c r="C357" s="21" t="s">
@@ -12591,14 +12523,14 @@
       <c r="J370" s="17">
         <v>3610988.6924000001</v>
       </c>
-      <c r="L370" s="25"/>
-      <c r="M370" s="25"/>
-      <c r="N370" s="25"/>
-      <c r="O370" s="25"/>
-      <c r="P370" s="25"/>
-      <c r="Q370" s="25"/>
-      <c r="R370" s="25"/>
-      <c r="S370" s="25"/>
+      <c r="L370" s="26"/>
+      <c r="M370" s="26"/>
+      <c r="N370" s="26"/>
+      <c r="O370" s="26"/>
+      <c r="P370" s="26"/>
+      <c r="Q370" s="26"/>
+      <c r="R370" s="26"/>
+      <c r="S370" s="26"/>
     </row>
     <row r="371" spans="3:19" ht="12.75" x14ac:dyDescent="0.2">
       <c r="C371" s="21" t="s">
@@ -13051,14 +12983,14 @@
       <c r="J384" s="17">
         <v>3757392.0140000004</v>
       </c>
-      <c r="L384" s="25"/>
-      <c r="M384" s="25"/>
-      <c r="N384" s="25"/>
-      <c r="O384" s="25"/>
-      <c r="P384" s="25"/>
-      <c r="Q384" s="25"/>
-      <c r="R384" s="25"/>
-      <c r="S384" s="25"/>
+      <c r="L384" s="26"/>
+      <c r="M384" s="26"/>
+      <c r="N384" s="26"/>
+      <c r="O384" s="26"/>
+      <c r="P384" s="26"/>
+      <c r="Q384" s="26"/>
+      <c r="R384" s="26"/>
+      <c r="S384" s="26"/>
     </row>
     <row r="385" spans="3:19" ht="12.75" x14ac:dyDescent="0.2">
       <c r="C385" s="21" t="s">
@@ -13511,14 +13443,14 @@
       <c r="J398" s="17">
         <v>3900345.2380000004</v>
       </c>
-      <c r="L398" s="25"/>
-      <c r="M398" s="25"/>
-      <c r="N398" s="25"/>
-      <c r="O398" s="25"/>
-      <c r="P398" s="25"/>
-      <c r="Q398" s="25"/>
-      <c r="R398" s="25"/>
-      <c r="S398" s="25"/>
+      <c r="L398" s="26"/>
+      <c r="M398" s="26"/>
+      <c r="N398" s="26"/>
+      <c r="O398" s="26"/>
+      <c r="P398" s="26"/>
+      <c r="Q398" s="26"/>
+      <c r="R398" s="26"/>
+      <c r="S398" s="26"/>
     </row>
     <row r="399" spans="3:19" ht="12.75" x14ac:dyDescent="0.2">
       <c r="C399" s="21" t="s">
@@ -13972,14 +13904,14 @@
         <v>3206833.645</v>
       </c>
       <c r="K412" s="7"/>
-      <c r="L412" s="25"/>
-      <c r="M412" s="25"/>
-      <c r="N412" s="25"/>
-      <c r="O412" s="25"/>
-      <c r="P412" s="25"/>
-      <c r="Q412" s="25"/>
-      <c r="R412" s="25"/>
-      <c r="S412" s="25"/>
+      <c r="L412" s="26"/>
+      <c r="M412" s="26"/>
+      <c r="N412" s="26"/>
+      <c r="O412" s="26"/>
+      <c r="P412" s="26"/>
+      <c r="Q412" s="26"/>
+      <c r="R412" s="26"/>
+      <c r="S412" s="26"/>
     </row>
     <row r="413" spans="3:19" ht="12.75" x14ac:dyDescent="0.2">
       <c r="C413" s="21" t="s">
@@ -14442,14 +14374,14 @@
         <v>3606958.7226859862</v>
       </c>
       <c r="K426" s="6"/>
-      <c r="L426" s="25"/>
-      <c r="M426" s="25"/>
-      <c r="N426" s="25"/>
-      <c r="O426" s="25"/>
-      <c r="P426" s="25"/>
-      <c r="Q426" s="25"/>
-      <c r="R426" s="25"/>
-      <c r="S426" s="25"/>
+      <c r="L426" s="26"/>
+      <c r="M426" s="26"/>
+      <c r="N426" s="26"/>
+      <c r="O426" s="26"/>
+      <c r="P426" s="26"/>
+      <c r="Q426" s="26"/>
+      <c r="R426" s="26"/>
+      <c r="S426" s="26"/>
     </row>
     <row r="427" spans="3:19" ht="12.75" x14ac:dyDescent="0.2">
       <c r="C427" s="21" t="s">
@@ -14916,14 +14848,14 @@
         <v>3888570.9300095243</v>
       </c>
       <c r="K440" s="6"/>
-      <c r="L440" s="25"/>
-      <c r="M440" s="25"/>
-      <c r="N440" s="25"/>
-      <c r="O440" s="25"/>
-      <c r="P440" s="25"/>
-      <c r="Q440" s="25"/>
-      <c r="R440" s="25"/>
-      <c r="S440" s="25"/>
+      <c r="L440" s="26"/>
+      <c r="M440" s="26"/>
+      <c r="N440" s="26"/>
+      <c r="O440" s="26"/>
+      <c r="P440" s="26"/>
+      <c r="Q440" s="26"/>
+      <c r="R440" s="26"/>
+      <c r="S440" s="26"/>
     </row>
     <row r="441" spans="3:19" ht="12.75" x14ac:dyDescent="0.2">
       <c r="C441" s="21" t="s">
@@ -15390,14 +15322,14 @@
         <v>3977360.585</v>
       </c>
       <c r="K454" s="6"/>
-      <c r="L454" s="25"/>
-      <c r="M454" s="25"/>
-      <c r="N454" s="25"/>
-      <c r="O454" s="25"/>
-      <c r="P454" s="25"/>
-      <c r="Q454" s="25"/>
-      <c r="R454" s="25"/>
-      <c r="S454" s="25"/>
+      <c r="L454" s="26"/>
+      <c r="M454" s="26"/>
+      <c r="N454" s="26"/>
+      <c r="O454" s="26"/>
+      <c r="P454" s="26"/>
+      <c r="Q454" s="26"/>
+      <c r="R454" s="26"/>
+      <c r="S454" s="26"/>
     </row>
     <row r="455" spans="3:19" ht="12.75" x14ac:dyDescent="0.2">
       <c r="C455" s="21" t="s">
@@ -15839,8 +15771,8 @@
       <c r="S467" s="3"/>
     </row>
     <row r="468" spans="3:19" ht="13.5" x14ac:dyDescent="0.2">
-      <c r="C468" s="20" t="s">
-        <v>21</v>
+      <c r="C468" s="20">
+        <v>2024</v>
       </c>
       <c r="D468" s="24">
         <v>765683.74</v>
@@ -16313,8 +16245,8 @@
       <c r="S481" s="3"/>
     </row>
     <row r="482" spans="3:19" ht="13.5" x14ac:dyDescent="0.2">
-      <c r="C482" s="20" t="s">
-        <v>22</v>
+      <c r="C482" s="20">
+        <v>2025</v>
       </c>
       <c r="D482" s="24">
         <v>787303.67000000016</v>
@@ -16788,28 +16720,28 @@
     </row>
     <row r="496" spans="3:19" ht="13.5" x14ac:dyDescent="0.2">
       <c r="C496" s="20" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D496" s="24">
-        <v>232507.33999999997</v>
+        <v>325114.33999999997</v>
       </c>
       <c r="E496" s="24">
-        <v>239755.66000000003</v>
+        <v>314127.57000000007</v>
       </c>
       <c r="F496" s="24">
-        <v>152769</v>
+        <v>243298</v>
       </c>
       <c r="G496" s="24">
-        <v>76857.11</v>
+        <v>84216.11</v>
       </c>
       <c r="H496" s="24">
-        <v>46423.880000000005</v>
+        <v>75659.16</v>
       </c>
       <c r="I496" s="24">
-        <v>310400.86800000002</v>
+        <v>461215.91</v>
       </c>
       <c r="J496" s="24">
-        <v>1058713.858</v>
+        <v>1503631.09</v>
       </c>
       <c r="K496" s="6"/>
       <c r="L496" s="3"/>
@@ -16825,25 +16757,25 @@
       <c r="C497" s="21" t="s">
         <v>0</v>
       </c>
-      <c r="D497" s="27">
+      <c r="D497" s="28">
         <v>59030.229999999996</v>
       </c>
-      <c r="E497" s="27">
+      <c r="E497" s="28">
         <v>94628.85</v>
       </c>
-      <c r="F497" s="27">
+      <c r="F497" s="28">
         <v>50403</v>
       </c>
-      <c r="G497" s="27">
+      <c r="G497" s="28">
         <v>8424</v>
       </c>
-      <c r="H497" s="27">
+      <c r="H497" s="28">
         <v>13745.490000000002</v>
       </c>
-      <c r="I497" s="27">
+      <c r="I497" s="28">
         <v>103548.052</v>
       </c>
-      <c r="J497" s="27">
+      <c r="J497" s="28">
         <v>329779.62199999997</v>
       </c>
       <c r="K497" s="6"/>
@@ -16860,25 +16792,25 @@
       <c r="C498" s="21" t="s">
         <v>1</v>
       </c>
-      <c r="D498" s="27">
+      <c r="D498" s="28">
         <v>49961.399999999994</v>
       </c>
-      <c r="E498" s="27">
+      <c r="E498" s="28">
         <v>37817.950000000004</v>
       </c>
-      <c r="F498" s="27">
+      <c r="F498" s="28">
         <v>27094</v>
       </c>
-      <c r="G498" s="27">
+      <c r="G498" s="28">
         <v>14712.72</v>
       </c>
-      <c r="H498" s="27">
+      <c r="H498" s="28">
         <v>10184.650000000001</v>
       </c>
-      <c r="I498" s="27">
+      <c r="I498" s="28">
         <v>68268.429999999993</v>
       </c>
-      <c r="J498" s="27">
+      <c r="J498" s="28">
         <v>208039.15</v>
       </c>
       <c r="K498" s="6"/>
@@ -16895,25 +16827,25 @@
       <c r="C499" s="21" t="s">
         <v>2</v>
       </c>
-      <c r="D499" s="27">
+      <c r="D499" s="28">
         <v>61476.22</v>
       </c>
-      <c r="E499" s="27">
+      <c r="E499" s="28">
         <v>51565.710000000006</v>
       </c>
-      <c r="F499" s="27">
+      <c r="F499" s="28">
         <v>36778</v>
       </c>
-      <c r="G499" s="27">
+      <c r="G499" s="28">
         <v>23254.86</v>
       </c>
-      <c r="H499" s="27">
+      <c r="H499" s="28">
         <v>10115.700000000001</v>
       </c>
-      <c r="I499" s="27">
+      <c r="I499" s="28">
         <v>76813.577000000005</v>
       </c>
-      <c r="J499" s="27">
+      <c r="J499" s="28">
         <v>260004.06699999998</v>
       </c>
       <c r="K499" s="6"/>
@@ -16927,28 +16859,28 @@
       <c r="S499" s="3"/>
     </row>
     <row r="500" spans="3:19" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="C500" s="22" t="s">
+      <c r="C500" s="21" t="s">
         <v>3</v>
       </c>
-      <c r="D500" s="29">
+      <c r="D500" s="28">
         <v>62039.49</v>
       </c>
-      <c r="E500" s="29">
+      <c r="E500" s="28">
         <v>55743.150000000009</v>
       </c>
-      <c r="F500" s="29">
+      <c r="F500" s="28">
         <v>38494</v>
       </c>
-      <c r="G500" s="29">
+      <c r="G500" s="28">
         <v>30465.53</v>
       </c>
-      <c r="H500" s="29">
+      <c r="H500" s="28">
         <v>12378.039999999999</v>
       </c>
-      <c r="I500" s="29">
+      <c r="I500" s="28">
         <v>61770.809000000001</v>
       </c>
-      <c r="J500" s="29">
+      <c r="J500" s="28">
         <v>260891.01900000003</v>
       </c>
       <c r="K500" s="6"/>
@@ -16962,31 +16894,120 @@
       <c r="S500" s="3"/>
     </row>
     <row r="501" spans="3:19" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="C501" s="28" t="s">
-        <v>23</v>
-      </c>
-      <c r="D501" s="2"/>
-      <c r="E501" s="2"/>
-      <c r="F501" s="2"/>
-      <c r="G501" s="2"/>
-      <c r="H501" s="2"/>
-      <c r="J501" s="2"/>
-    </row>
-    <row r="502" spans="3:19" x14ac:dyDescent="0.2">
-      <c r="C502" s="28" t="s">
-        <v>26</v>
-      </c>
-      <c r="I502" s="4"/>
-    </row>
-    <row r="503" spans="3:19" x14ac:dyDescent="0.2">
-      <c r="C503" s="9"/>
-      <c r="D503" s="26"/>
-      <c r="E503" s="26"/>
-      <c r="F503" s="26"/>
-      <c r="G503" s="26"/>
-      <c r="H503" s="26"/>
-      <c r="I503" s="26"/>
-      <c r="J503" s="26"/>
+      <c r="C501" s="21" t="s">
+        <v>25</v>
+      </c>
+      <c r="D501" s="28">
+        <v>49421.55</v>
+      </c>
+      <c r="E501" s="28">
+        <v>27464.879999999997</v>
+      </c>
+      <c r="F501" s="28">
+        <v>38715</v>
+      </c>
+      <c r="G501" s="28">
+        <v>7359</v>
+      </c>
+      <c r="H501" s="28">
+        <v>13502.15</v>
+      </c>
+      <c r="I501" s="28">
+        <v>86308.142999999996</v>
+      </c>
+      <c r="J501" s="28">
+        <v>222770.723</v>
+      </c>
+      <c r="K501" s="6"/>
+      <c r="L501" s="3"/>
+      <c r="M501" s="3"/>
+      <c r="N501" s="3"/>
+      <c r="O501" s="3"/>
+      <c r="P501" s="3"/>
+      <c r="Q501" s="3"/>
+      <c r="R501" s="3"/>
+      <c r="S501" s="3"/>
+    </row>
+    <row r="502" spans="3:19" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="C502" s="21" t="s">
+        <v>5</v>
+      </c>
+      <c r="D502" s="28">
+        <v>43185.450000000004</v>
+      </c>
+      <c r="E502" s="28">
+        <v>46907.03</v>
+      </c>
+      <c r="F502" s="28">
+        <v>51814</v>
+      </c>
+      <c r="G502" s="28">
+        <v>0</v>
+      </c>
+      <c r="H502" s="28">
+        <v>15733.129999999997</v>
+      </c>
+      <c r="I502" s="28">
+        <v>64506.89899999999</v>
+      </c>
+      <c r="J502" s="28">
+        <v>222146.50900000002</v>
+      </c>
+      <c r="K502" s="6"/>
+      <c r="L502" s="3"/>
+      <c r="M502" s="3"/>
+      <c r="N502" s="3"/>
+      <c r="O502" s="3"/>
+      <c r="P502" s="3"/>
+      <c r="Q502" s="3"/>
+      <c r="R502" s="3"/>
+      <c r="S502" s="3"/>
+    </row>
+    <row r="503" spans="3:19" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="C503" s="22"/>
+      <c r="D503" s="25"/>
+      <c r="E503" s="25"/>
+      <c r="F503" s="25"/>
+      <c r="G503" s="25"/>
+      <c r="H503" s="25"/>
+      <c r="I503" s="25"/>
+      <c r="J503" s="25"/>
+      <c r="K503" s="6"/>
+      <c r="L503" s="3"/>
+      <c r="M503" s="3"/>
+      <c r="N503" s="3"/>
+      <c r="O503" s="3"/>
+      <c r="P503" s="3"/>
+      <c r="Q503" s="3"/>
+      <c r="R503" s="3"/>
+      <c r="S503" s="3"/>
+    </row>
+    <row r="504" spans="3:19" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="C504" s="9" t="s">
+        <v>22</v>
+      </c>
+      <c r="D504" s="2"/>
+      <c r="E504" s="2"/>
+      <c r="F504" s="2"/>
+      <c r="G504" s="2"/>
+      <c r="H504" s="2"/>
+      <c r="J504" s="2"/>
+    </row>
+    <row r="505" spans="3:19" x14ac:dyDescent="0.2">
+      <c r="C505" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="I505" s="4"/>
+    </row>
+    <row r="506" spans="3:19" x14ac:dyDescent="0.2">
+      <c r="C506" s="9"/>
+      <c r="D506" s="27"/>
+      <c r="E506" s="27"/>
+      <c r="F506" s="27"/>
+      <c r="G506" s="27"/>
+      <c r="H506" s="27"/>
+      <c r="I506" s="27"/>
+      <c r="J506" s="27"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>